<commit_message>
Stage 8 review fixes: E-004
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/WX4/WA-2015-137/Results/Approved/WX4_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
+++ b/output/archive/WestravelleData/Stability/WX4/WA-2015-137/Results/Approved/WX4_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
@@ -172,9 +172,9 @@
     <author>Alice Penrose</author>
   </authors>
   <commentList>
-    <comment ref="C5" authorId="0" shapeId="0">
+    <comment ref="B3" authorId="0" shapeId="0">
       <text>
-        <t>Units on the sequence sheet to be aligned with the batch card at the next revision.</t>
+        <t>Retain source deviation references with the sequence sheets.</t>
       </text>
     </comment>
   </commentList>
@@ -624,7 +624,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Eighteen-month ICH stability of WX-4 tablets in the two packs under test, with the HPLC assay and related-substances method qualified before the first pull. Interim review completed 22 Apr 2016.</t>
+          <t>Eighteen-month ICH stability of WX-4 tablets with assay and related-substances qualification. Interim review completed 22 Apr 2016.</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Assay as % label claim (HPLC). Impurities as % area. Water by Karl Fischer. Pack A is the standard blister; pack B is the higher-barrier blister.</t>
+          <t>Assay as % label claim (HPLC). Impurities as % area. Water by Karl Fischer. The table is organised by storage condition, not by packaging presentation; packaging identities and comparison records remain on the batch card. Time zero is one initial analysis shared by all storage conditions; repeated initial rows do not represent separate pulls.</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1550,162 +1550,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Units are recorded as written on the batch card. Concentrations are for the working solutions used in the sequences.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Preparation details</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Refer to the batch card for standard, sample and impurity-reference preparations.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Solution</t>
+          <t>Concentration notation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Nominal concentration</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Units as written</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Storage</t>
+          <t>Stock entries use mg/mL; working-solution entries use mg/ml. Refer to the preparation record for concentrations.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Standard stock</t>
+          <t>Storage and use periods</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1.0 mg/mL in diluent</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>mg/mL</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Refrigerated, 7 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Working standard</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>0.10 mg/ml</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>mg/ml</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Prepared fresh each day</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Impurity spike, Imp A</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>5 µM</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>µM</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Refrigerated, protected from light</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Impurity spike, Imp B</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>50 nM</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>nM</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Refrigerated, protected from light</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Sample solution</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>0.5 mg/mL</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>mg/mL</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Prepared on the day of analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Low-level check</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>200 ng/ml</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>ng/ml</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Prepared fresh each day</t>
+          <t>Refer to the preparation record; this summary does not assign solution expiry.</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1733,78 +1619,57 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Deviation notes</t>
+          <t>Deviation notes and reporting interval</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ref</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Raised</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Record</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DN-01</t>
+          <t>Deviation / repeat history</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>14 Apr 2016</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Eighteen-month pack B pull logged against the wrong chamber position. Position corrected in LIMS and the sample confirmed by the chamber log.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Closed 18 Apr 2016</t>
+          <t>Refer to the batch card and approved sequence sheets.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DN-02</t>
+          <t>Reporting interval</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>19 Dec 2016</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Impurity spike solution prepared at 5 µM instead of the 5 nM written on the sequence sheet. Spike remade and the affected run repeated.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Closed 21 Dec 2016</t>
+          <t>Long-term and intermediate pulls extend to the final reported timepoint; accelerated pulls stop at six months.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Packaging decision</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Wexanthel adopted the higher-barrier blister following the packaging-dependent impurity trend. The condition table does not quantify that comparison.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>